<commit_message>
Importmallar: granskningsfynd — tomma cellers undantag, valuta på nya katalograder, varning för hoppad Orderkvantitet, resursnummer fylls ut, textformat i mallen, rättade förklaringar; CLAUDE.md och TODO
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HZtLXoU1UGUT8jwRKLYmYe
</commit_message>
<xml_diff>
--- a/apps/web/public/importmallar/importmall-artiklar.xlsx
+++ b/apps/web/public/importmallar/importmall-artiklar.xlsx
@@ -22,7 +22,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Obligatorisk. Artikelns unika nummer, max 50 tecken. Finns numret redan uppdateras artikeln, annars skapas en ny. Textformatera kolumnen i Excel så att inledande nollor behålls.</t>
+          <t xml:space="preserve">Obligatorisk. Artikelns unika nummer, max 50 tecken. Finns numret redan uppdateras artikeln, annars skapas en ny. Mallens kolumn är textformaterad så att inledande nollor behålls.</t>
         </r>
       </text>
     </comment>
@@ -142,7 +142,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Saldo i grundenhet där behovsberäkningen föreslår påfyllnad, decimalkomma eller punkt, aldrig negativt. 0 betyder ingen beställningspunkt och tömmer fältet; tom cell lämnar det orört.</t>
+          <t xml:space="preserve">Nivån i grundenhet som behovsberäkningen fyller upp till: den jämför med det beräknade saldot (lager + inkommande − behov) och föreslår skillnaden när saldot ligger under. Decimalkomma eller punkt, aldrig negativ. 0 betyder ingen beställningspunkt och tömmer fältet; tom cell lämnar det orört.</t>
         </r>
       </text>
     </comment>
@@ -154,7 +154,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Fast orderstorlek i grundenhet — förslag rundas upp till en multipel av den. Importeras bara när Partiformningsregel är Fast orderstorlek (eller den kolumnen inte är mappad). 0 tömmer fältet; tom cell lämnar det orört.</t>
+          <t xml:space="preserve">Fast orderstorlek i grundenhet — förslag rundas upp till en multipel av den. Importeras bara när Partiformningsregel är Fast orderstorlek eller den kolumnen saknas; finns kolumnen men är regeln något annat eller tom hoppas Orderkvantitet över med en varning. 0 tömmer fältet; tom cell lämnar det orört.</t>
         </r>
       </text>
     </comment>
@@ -178,7 +178,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Lagras inte — styr bara om Orderkvantitet läses: Fast orderstorlek betyder att kvantiteten importeras, allt annat (t.ex. Mot behov) att den hoppas över på raden.</t>
+          <t xml:space="preserve">Lagras inte — styr bara om Orderkvantitet läses: Fast orderstorlek betyder att kvantiteten importeras, allt annat (t.ex. Mot behov) och tom cell att den hoppas över på raden, med en varning. Ta bort kolumnen för att alltid läsa Orderkvantitet.</t>
         </r>
       </text>
     </comment>
@@ -221,7 +221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -230,6 +230,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -241,11 +242,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="1" max="1" width="17" customWidth="1" style="4"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1" style="4"/>
+    <col min="5" max="5" width="22" customWidth="1" style="4"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
@@ -362,88 +363,73 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kolumner du inte behöver kan tas bort eller lämnas tomma, och kolumnernas ordning spelar ingen roll.</t>
+          <t xml:space="preserve">Ta bort kolumner du inte använder. Kolumnernas ordning spelar ingen roll.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t xml:space="preserve">En tom cell lämnar normalt värdet orört på en befintlig post, utom i kolumner där tomt betyder något: Huvudleverantör och Staffel: från antal/Staffel: pris (Inköpspriser), Partiformningsregel (Artiklar) samt Kalkyl och Tidsenhet med Uppdatera befintliga operationer (Operationer). Vad tomt betyder står vid varje kolumn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t xml:space="preserve">Tal skrivs med decimalkomma eller punkt. Obligatoriska kolumner måste finnas med och vara ifyllda på varje rad.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Kolumn</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Obligatorisk</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Förklaring</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Exempel</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Artikelnummer</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ja</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Artikelns unika nummer, max 50 tecken. Finns numret redan uppdateras artikeln, annars skapas en ny. Textformatera kolumnen i Excel så att inledande nollor behålls.</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SB-1200</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Benämning</t>
+          <t xml:space="preserve">Artikelnummer</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nej</t>
+          <t xml:space="preserve">Ja</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Artikelns namn, max 255 tecken. Krävs för nya artiklar. Tom cell lämnar fältet orört på en befintlig post.</t>
+          <t xml:space="preserve">Artikelns unika nummer, max 50 tecken. Finns numret redan uppdateras artikeln, annars skapas en ny. Mallens kolumn är textformaterad så att inledande nollor behålls.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diskbänk 1200 mm, rostfri</t>
+          <t xml:space="preserve">SB-1200</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Artikeltyp</t>
+          <t xml:space="preserve">Benämning</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -453,19 +439,19 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tillverkad (även M), Köpt (även P eller K), Tjänst (även Lego) eller Fiktiv (även F) — Fiktiv ger en tillverkad fantomartikel. Tom cell ger guidens Standardtyp för nya artiklar. Typen och fantomflaggan ändras aldrig på befintliga artiklar — en avvikelse ger en varning.</t>
+          <t xml:space="preserve">Artikelns namn, max 255 tecken. Krävs för nya artiklar. Tom cell lämnar fältet orört på en befintlig post.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tillverkad</t>
+          <t xml:space="preserve">Diskbänk 1200 mm, rostfri</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enhet</t>
+          <t xml:space="preserve">Artikeltyp</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -475,19 +461,19 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grundenhetens kod, max 20 tecken (t.ex. st, kg, m). En okänd kod skapas i enhetsregistret med koden som namn; tom cell ger st för nya artiklar. Grundenheten ändras aldrig på befintliga artiklar.</t>
+          <t xml:space="preserve">Tillverkad (även M), Köpt (även P eller K), Tjänst (även Lego) eller Fiktiv (även F) — Fiktiv ger en tillverkad fantomartikel. Tom cell ger guidens Standardtyp för nya artiklar. Typen och fantomflaggan ändras aldrig på befintliga artiklar — en avvikelse ger en varning.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">st</t>
+          <t xml:space="preserve">Tillverkad</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Artikelgrupp (kod)</t>
+          <t xml:space="preserve">Enhet</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -497,19 +483,19 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Artikelgruppens kod, 3–4 siffror. En kod som saknas i registret skapas med koden som namn. Tom cell lämnar fältet orört på en befintlig post.</t>
+          <t xml:space="preserve">Grundenhetens kod, max 20 tecken (t.ex. st, kg, m). En okänd kod skapas i enhetsregistret med koden som namn; tom cell ger st för nya artiklar. Grundenheten ändras aldrig på befintliga artiklar.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">300</t>
+          <t xml:space="preserve">st</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Standardpris</t>
+          <t xml:space="preserve">Artikelgrupp (kod)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -519,19 +505,19 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Standardkostnad per grundenhet i SEK, decimalkomma eller punkt, aldrig negativ (t.ex. 1 250,50). Tom cell lämnar fältet orört; ett annat värde än det sparade uppdaterar artikeln.</t>
+          <t xml:space="preserve">Artikelgruppens kod, 3–4 siffror. En kod som saknas i registret skapas med koden som namn. Tom cell lämnar fältet orört på en befintlig post.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1250,50</t>
+          <t xml:space="preserve">300</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vikt (kg)</t>
+          <t xml:space="preserve">Standardpris</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -541,19 +527,19 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vikt i kilogram per grundenhet, decimalkomma eller punkt, aldrig negativ. Tom cell lämnar fältet orört på en befintlig post.</t>
+          <t xml:space="preserve">Standardkostnad per grundenhet i SEK, decimalkomma eller punkt, aldrig negativ (t.ex. 1 250,50). Tom cell lämnar fältet orört; ett annat värde än det sparade uppdaterar artikeln.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">18,5</t>
+          <t xml:space="preserve">1250,50</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ytbehandling</t>
+          <t xml:space="preserve">Vikt (kg)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -563,19 +549,19 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fritext, max 200 tecken. Tom cell lämnar fältet orört på en befintlig post.</t>
+          <t xml:space="preserve">Vikt i kilogram per grundenhet, decimalkomma eller punkt, aldrig negativ. Tom cell lämnar fältet orört på en befintlig post.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Borstad</t>
+          <t xml:space="preserve">18,5</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Färg</t>
+          <t xml:space="preserve">Ytbehandling</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -590,14 +576,14 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rostfri</t>
+          <t xml:space="preserve">Borstad</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aktiv</t>
+          <t xml:space="preserve">Färg</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -607,19 +593,19 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ja/Nej, 1/0 eller true/false. Tom cell betyder aktiv för nya artiklar och lämnar befintliga orörda.</t>
+          <t xml:space="preserve">Fritext, max 200 tecken. Tom cell lämnar fältet orört på en befintlig post.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ja</t>
+          <t xml:space="preserve">Rostfri</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Beställningspunkt</t>
+          <t xml:space="preserve">Aktiv</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -629,19 +615,19 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Saldo i grundenhet där behovsberäkningen föreslår påfyllnad, decimalkomma eller punkt, aldrig negativt. 0 betyder ingen beställningspunkt och tömmer fältet; tom cell lämnar det orört.</t>
+          <t xml:space="preserve">Ja/Nej, 1/0 eller true/false. Tom cell betyder aktiv för nya artiklar och lämnar befintliga orörda.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">Ja</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Orderkvantitet</t>
+          <t xml:space="preserve">Beställningspunkt</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -651,19 +637,19 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fast orderstorlek i grundenhet — förslag rundas upp till en multipel av den. Importeras bara när Partiformningsregel är Fast orderstorlek (eller den kolumnen inte är mappad). 0 tömmer fältet; tom cell lämnar det orört.</t>
+          <t xml:space="preserve">Nivån i grundenhet som behovsberäkningen fyller upp till: den jämför med det beräknade saldot (lager + inkommande − behov) och föreslår skillnaden när saldot ligger under. Decimalkomma eller punkt, aldrig negativ. 0 betyder ingen beställningspunkt och tömmer fältet; tom cell lämnar det orört.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">25</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Avrundning</t>
+          <t xml:space="preserve">Orderkvantitet</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -673,32 +659,54 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Steg i grundenhet som orderantal rundas upp till, större än 0 och högst 3 decimaler (fler avrundas med en varning). 0 tömmer fältet; tom cell lämnar det orört.</t>
+          <t xml:space="preserve">Fast orderstorlek i grundenhet — förslag rundas upp till en multipel av den. Importeras bara när Partiformningsregel är Fast orderstorlek eller den kolumnen saknas; finns kolumnen men är regeln något annat eller tom hoppas Orderkvantitet över med en varning. 0 tömmer fältet; tom cell lämnar det orört.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">25</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Avrundning</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Steg i grundenhet som orderantal rundas upp till, större än 0 och högst 3 decimaler (fler avrundas med en varning). 0 tömmer fältet; tom cell lämnar det orört.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Partiformningsregel</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nej</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lagras inte — styr bara om Orderkvantitet läses: Fast orderstorlek betyder att kvantiteten importeras, allt annat (t.ex. Mot behov) att den hoppas över på raden.</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lagras inte — styr bara om Orderkvantitet läses: Fast orderstorlek betyder att kvantiteten importeras, allt annat (t.ex. Mot behov) och tom cell att den hoppas över på raden, med en varning. Ta bort kolumnen för att alltid läsa Orderkvantitet.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Fast orderstorlek</t>
         </is>

</xml_diff>

<commit_message>
Artikelimporten: Artikelrevision, Ritningsnummer och Ritningsrevision
- Tre nya fält i artikelimporten och mallen. Artikelrevision blir
  artikelns aktiva revision (läggs till om den saknas, den tidigare blir
  inaktiv; förhandsgranskningen varnar när den aktiva byts och en
  oförändrad revision skrivs inte). Ritningsnummer läggs till om artikeln
  saknar det. Ritningsrevision blir aktiv revision för ritningsnumret på
  samma rad och kräver det (annars radfel). Importen tar aldrig bort
  något och är idempotent.
- Skrivningen är lövfilen import/repository/article-revisions.ts
  (applyImportedRevisions i executeArticlePlans transaktion, ren
  revisionChanges); articlesByNumber bär activeRevision.
- Fälthjälpen, importmall-artiklar.xlsx och kapitlet Importmallar
  omgenererade; manualens Importera artiklar och Revisioner uppdaterade.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HZtLXoU1UGUT8jwRKLYmYe
</commit_message>
<xml_diff>
--- a/apps/web/public/importmallar/importmall-artiklar.xlsx
+++ b/apps/web/public/importmallar/importmall-artiklar.xlsx
@@ -179,6 +179,42 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">Lagras inte — styr bara om Orderkvantitet läses: Fast orderstorlek betyder att kvantiteten importeras, allt annat (t.ex. Mot behov) och tom cell att den hoppas över på raden, med en varning. Ta bort kolumnen för att alltid läsa Orderkvantitet.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Artikelns aktiva revision, max 20 tecken. Saknar artikeln revisionen läggs den till; den blir aktiv och den tidigare aktiva ligger kvar som inaktiv (förhandsgranskningen varnar när den aktiva byts). Importen tar aldrig bort en revision. Tom cell lämnar revisionerna orörda.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Ett ritningsnummer på artikeln, max 50 tecken. Saknar artikeln numret läggs det till — artikelns andra ritningsnummer ligger kvar, importen tar aldrig bort något. Varje rad ger ett ritningsnummer, och ett artikelnummer får bara förekomma en gång per fil — har en artikel flera ritningar importeras de övriga i en ny körning. Tom cell lämnar ritningarna orörda.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Den aktiva revisionen för ritningsnumret på samma rad, max 20 tecken — kräver Ritningsnummer på raden. Saknas revisionen läggs den till; den blir aktiv och den tidigare aktiva ligger kvar som inaktiv. Tom cell lämnar ritningens revisioner orörda.</t>
         </r>
       </text>
     </comment>
@@ -256,6 +292,9 @@
     <col min="12" max="12" width="18" customWidth="1"/>
     <col min="13" max="13" width="14" customWidth="1"/>
     <col min="14" max="14" width="23" customWidth="1"/>
+    <col min="15" max="15" width="19" customWidth="1" style="4"/>
+    <col min="16" max="16" width="18" customWidth="1" style="4"/>
+    <col min="17" max="17" width="20" customWidth="1" style="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -327,6 +366,21 @@
       <c r="N1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Partiformningsregel</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Artikelrevision</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ritningsnummer</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ritningsrevision</t>
         </is>
       </c>
     </row>
@@ -712,6 +766,72 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Artikelrevision</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Artikelns aktiva revision, max 20 tecken. Saknar artikeln revisionen läggs den till; den blir aktiv och den tidigare aktiva ligger kvar som inaktiv (förhandsgranskningen varnar när den aktiva byts). Importen tar aldrig bort en revision. Tom cell lämnar revisionerna orörda.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ritningsnummer</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ett ritningsnummer på artikeln, max 50 tecken. Saknar artikeln numret läggs det till — artikelns andra ritningsnummer ligger kvar, importen tar aldrig bort något. Varje rad ger ett ritningsnummer, och ett artikelnummer får bara förekomma en gång per fil — har en artikel flera ritningar importeras de övriga i en ny körning. Tom cell lämnar ritningarna orörda.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R-63010</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ritningsrevision</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Den aktiva revisionen för ritningsnumret på samma rad, max 20 tecken — kräver Ritningsnummer på raden. Saknas revisionen läggs den till; den blir aktiv och den tidigare aktiva ligger kvar som inaktiv. Tom cell lämnar ritningens revisioner orörda.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Säkerhetslager och Styrning på artikeln
- articles.safety_stock och stock_controlled (0163). Behovsberäkningen föreslår när det beräknade saldot faller under det största av beställningspunkt och säkerhetslager och fyller upp till den nivån (sedan orderkvantitet och avrundning som förut). Styrning Lagerstyrd/Orderstyrd är information.
- Lager-flikens Planering, behovsberäkningens BP / SL-kolumn, Kopiera från → Information och artikelimportens Säkerhetslager/Styrning ur planeringsexporten.

Manual, importmall och tester uppdaterade.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013pvWaFZiioxpDd9AVeYPCR
</commit_message>
<xml_diff>
--- a/apps/web/public/importmallar/importmall-artiklar.xlsx
+++ b/apps/web/public/importmallar/importmall-artiklar.xlsx
@@ -214,11 +214,35 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
+          <t xml:space="preserve">Lägsta beräknade saldo i grundenheten, decimalkomma eller punkt, aldrig negativt. Faller saldot under det föreslår behovsberäkningen påfyllning upp till säkerhetslagret. 0 tömmer fältet. Tom cell lämnar fältet orört på en befintlig post.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Lagerstyrd eller Orderstyrd — sparas som information på Lager-flikens planering. Tom cell lämnar fältet orört på en befintlig post.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
           <t xml:space="preserve">Artikelns aktiva revision, max 20 tecken. Saknar artikeln revisionen läggs den till; den blir aktiv och den tidigare aktiva ligger kvar som inaktiv (förhandsgranskningen varnar när den aktiva byts). Importen tar aldrig bort en revision. Tom cell lämnar revisionerna orörda.</t>
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="0">
+    <comment ref="T1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -230,7 +254,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="0">
+    <comment ref="U1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -242,7 +266,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="0">
+    <comment ref="V1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -254,7 +278,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U1" authorId="0">
+    <comment ref="W1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -342,11 +366,13 @@
     <col min="14" max="14" width="18" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
     <col min="16" max="16" width="23" customWidth="1"/>
-    <col min="17" max="17" width="19" customWidth="1" style="4"/>
-    <col min="18" max="18" width="18" customWidth="1" style="4"/>
-    <col min="19" max="19" width="20" customWidth="1" style="4"/>
-    <col min="20" max="20" width="25" customWidth="1"/>
-    <col min="21" max="21" width="21" customWidth="1" style="4"/>
+    <col min="17" max="17" width="18" customWidth="1"/>
+    <col min="18" max="18" width="14" customWidth="1"/>
+    <col min="19" max="19" width="19" customWidth="1" style="4"/>
+    <col min="20" max="20" width="18" customWidth="1" style="4"/>
+    <col min="21" max="21" width="20" customWidth="1" style="4"/>
+    <col min="22" max="22" width="25" customWidth="1"/>
+    <col min="23" max="23" width="21" customWidth="1" style="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -432,25 +458,35 @@
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Säkerhetslager</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Styrning</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Artikelrevision</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Ritningsnummer</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Ritningsrevision</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Antal per förpackning</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Leverantörsnummer</t>
         </is>
@@ -885,7 +921,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Artikelrevision</t>
+          <t xml:space="preserve">Säkerhetslager</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -895,19 +931,19 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Artikelns aktiva revision, max 20 tecken. Saknar artikeln revisionen läggs den till; den blir aktiv och den tidigare aktiva ligger kvar som inaktiv (förhandsgranskningen varnar när den aktiva byts). Importen tar aldrig bort en revision. Tom cell lämnar revisionerna orörda.</t>
+          <t xml:space="preserve">Lägsta beräknade saldo i grundenheten, decimalkomma eller punkt, aldrig negativt. Faller saldot under det föreslår behovsberäkningen påfyllning upp till säkerhetslagret. 0 tömmer fältet. Tom cell lämnar fältet orört på en befintlig post.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">20</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ritningsnummer</t>
+          <t xml:space="preserve">Styrning</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -917,19 +953,19 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ett ritningsnummer på artikeln, max 50 tecken. Saknar artikeln numret läggs det till — artikelns andra ritningsnummer ligger kvar, importen tar aldrig bort något. Varje rad ger ett ritningsnummer, och ett artikelnummer får bara förekomma en gång per fil — har en artikel flera ritningar importeras de övriga i en ny körning. Tom cell lämnar ritningarna orörda.</t>
+          <t xml:space="preserve">Lagerstyrd eller Orderstyrd — sparas som information på Lager-flikens planering. Tom cell lämnar fältet orört på en befintlig post.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">R-63010</t>
+          <t xml:space="preserve">Lagerstyrd</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ritningsrevision</t>
+          <t xml:space="preserve">Artikelrevision</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -939,19 +975,19 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Den aktiva revisionen för ritningsnumret på samma rad, max 20 tecken — kräver Ritningsnummer på raden. Saknas revisionen läggs den till; den blir aktiv och den tidigare aktiva ligger kvar som inaktiv. Tom cell lämnar ritningens revisioner orörda.</t>
+          <t xml:space="preserve">Artikelns aktiva revision, max 20 tecken. Saknar artikeln revisionen läggs den till; den blir aktiv och den tidigare aktiva ligger kvar som inaktiv (förhandsgranskningen varnar när den aktiva byts). Importen tar aldrig bort en revision. Tom cell lämnar revisionerna orörda.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Antal per förpackning</t>
+          <t xml:space="preserve">Ritningsnummer</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -961,32 +997,76 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hur många av artikelns grundenhet som ryms i en förpackning (Inköp-fliken). Decimalkomma eller punkt, högst 4 decimaler — fler avrundas med en varning. 0 tömmer fältet. Tom cell lämnar fältet orört på en befintlig post.</t>
+          <t xml:space="preserve">Ett ritningsnummer på artikeln, max 50 tecken. Saknar artikeln numret läggs det till — artikelns andra ritningsnummer ligger kvar, importen tar aldrig bort något. Varje rad ger ett ritningsnummer, och ett artikelnummer får bara förekomma en gång per fil — har en artikel flera ritningar importeras de övriga i en ny körning. Tom cell lämnar ritningarna orörda.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">25</t>
+          <t xml:space="preserve">R-63010</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Ritningsrevision</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Den aktiva revisionen för ritningsnumret på samma rad, max 20 tecken — kräver Ritningsnummer på raden. Saknas revisionen läggs den till; den blir aktiv och den tidigare aktiva ligger kvar som inaktiv. Tom cell lämnar ritningens revisioner orörda.</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Antal per förpackning</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hur många av artikelns grundenhet som ryms i en förpackning (Inköp-fliken). Decimalkomma eller punkt, högst 4 decimaler — fler avrundas med en varning. 0 tömmer fältet. Tom cell lämnar fältet orört på en befintlig post.</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Leverantörsnummer</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nej</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Artikelns förvalda leverantör på Inköp-fliken. Leverantören måste finnas i leverantörsregistret — importera leverantörerna först. Har artikeln ingen rad för leverantören läggs en till utan pris (priserna kommer med inköpsprislistan); den tidigare förvalda leverantören blir kvar men inte förvald. Tom cell lämnar leverantörerna orörda.</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">20015</t>
         </is>

</xml_diff>